<commit_message>
Abu Ghazi Village: 250k refinance scenarios and study addendum
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SHa6crvVEuPcYfhvw5C66Y
</commit_message>
<xml_diff>
--- a/feasibility-study-team-of-agents/studies/abu-ghazi-village/model/AGV-financial-model.xlsx
+++ b/feasibility-study-team-of-agents/studies/abu-ghazi-village/model/AGV-financial-model.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Funding options" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Gallery scenarios" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Stress tests" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Refinance 140k" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="116">
   <si>
     <t xml:space="preserve">Input</t>
   </si>
@@ -346,6 +347,33 @@
   </si>
   <si>
     <t xml:space="preserve">Rents -20% (vacancy + discounts) and POS -30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1 250k CBJ sectors programme @3.25%, 12m grace + 108</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2 305k (140k refi + 165k new) CBJ @3.25%, 12m grace + 108</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3 110k CBJ @3.25% + 140k refi commercial @8.5% 10y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4 110k CBJ @3.25% + 140k refi Islamic @7% 15y (12m grace + 168)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5 RECOMMENDED if 250k: one 250k Islamic diminishing musharaka/ijara @7% 15y (12m grace + 168)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5s R5 with revenue -10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R6 250k commercial @8.5% 15y (12m grace + 168)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R7 305k: 165k CBJ + 140k refi Islamic @7% 15y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap: 205k CBJ @3.25% 10y (DSCR ~1.25 limit)</t>
   </si>
 </sst>
 </file>
@@ -7516,4 +7544,616 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:S10"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="O1" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="P1" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q1" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="R1" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="S1" s="0" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>2672.94792027257</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>1.02340784177696</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>1.02340784177696</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>1.09143792230849</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>1.14238944464576</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>43937.4778</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>46803.3753894351</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>3.37642803692308</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>1.02340784177696</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>1.05835075412957</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>1.06998824665599</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>1.08174889028339</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>1.09363247388494</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>1.10563871563042</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>1.11776725986846</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <v>1.1300176739009</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>1.14238944464576</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>305000</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>3260.99646273253</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0.847589856624582</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0.847589856624582</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0.899453469116443</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0.937011751376776</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>7096.23459245909</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>57100.1179751107</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>2.80362953846154</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0.847589856624582</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0.875329860159262</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0.883937313896171</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>0.892614983198843</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>0.901361681342834</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>0.910176130210648</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>0.919056956633093</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>0.928002688605778</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.937011751376776</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>3035.20646370714</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0.940448344437678</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0.940448344437678</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0.98504285259603</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>1.00978678425537</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>32595.7792915759</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>93277.2980803697</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>1.86775300807755</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0.940448344437678</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>0.968432935945745</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0.975510618305302</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>0.98227534663623</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0.988685030733057</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0.994693660582234</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>1.00025095757818</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>1.00530199489048</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>1.00978678425537</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>2485.65784343246</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1.13577612141075</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>1.13577612141075</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>1.20787812112457</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>1.26015731915948</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>39737.4778</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>97961.4760064849</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>2.12960581682243</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>1.13577612141075</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>1.17340244418782</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>1.18585262806213</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>1.19830835134258</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>1.21075618113489</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>1.22318152082184</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>1.23556852369249</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>1.24790000030919</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>1.26015731915948</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>2338.50135448666</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>1.23669240594029</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>1.23669240594029</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>1.31245133584937</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>1.3659228997272</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>36437.4778</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>138157.12649131</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>1.67477016</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>1.23669240594029</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>1.27672865980099</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>1.28990870971549</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>1.30298867371821</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>1.31594324464169</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>1.32874496997097</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>1.34136409070437</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>1.35376836842511</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>1.3659228997272</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>2338.50135448666</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>1.0073179917223</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>1.0073179917223</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>1.03814431685088</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>1.0643940972501</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>29549.6039</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>138157.12649131</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>1.28117736571429</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>1.0073179917223</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>1.01747078774397</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>1.02500711595283</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>1.03231672688785</v>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>1.03937136804651</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>1.04614057029082</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>1.05259148491096</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>1.0586887088526</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <v>1.0643940972501</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>2549.79633781845</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1.15854384275926</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>1.15854384275926</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>1.22475457139906</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>1.26880558856876</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>33437.4778</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>170908.093412315</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>1.41451660235294</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>1.15854384275926</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>1.19480032098096</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>1.20630227105639</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>1.21757165696192</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>1.22856639306385</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>1.23924029271305</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>1.2495426982657</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>1.25941807822167</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>1.26880558856876</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>305000</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>3073.70638589242</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0.927747197874385</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0.927747197874385</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0.981918636137919</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>1.01973449880731</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>31089.088561018</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>108258.218592161</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>1.90212549381698</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>0.927747197874385</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>0.957218338399617</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>0.966298373523007</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>0.975350287971057</v>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>0.984362143338596</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>0.99332102465907</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>1.00221296938751</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>1.01102289128072</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>1.01973449880731</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>205000</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>2191.81729462351</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1.23743017847021</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>1.23743017847021</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>1.32513961810102</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>1.39239466328141</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>45107.4778</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>38378.7678193368</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>4.07369272795497</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>1.23743017847021</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>1.28114115499366</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>1.29646709828601</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>1.31198063083642</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>1.32768272910804</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>1.34357432404606</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>1.35965629861838</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>1.37592948526901</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>1.39239466328141</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>